<commit_message>
basic_pipeline benchmarking done (former modular_pipeline)
</commit_message>
<xml_diff>
--- a/evaluation_metrics_reports/final_benchmark_report.xlsx
+++ b/evaluation_metrics_reports/final_benchmark_report.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,10 +468,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>11.94429165774526</v>
+        <v>11.68721463812928</v>
       </c>
       <c r="C2" t="n">
-        <v>3.73015873015873</v>
+        <v>3.809523809523809</v>
       </c>
       <c r="D2" t="n">
         <v>301.8271484375</v>
@@ -480,7 +480,7 @@
         <v>492.5759439468384</v>
       </c>
       <c r="F2" t="n">
-        <v>25.73015873015873</v>
+        <v>25.80952380952381</v>
       </c>
     </row>
     <row r="3">
@@ -490,10 +490,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>10.02702773950104</v>
+        <v>9.611612084841873</v>
       </c>
       <c r="C3" t="n">
-        <v>10.16319444444444</v>
+        <v>10.11458333333333</v>
       </c>
       <c r="D3" t="n">
         <v>301.8271484375</v>
@@ -502,7 +502,51 @@
         <v>492.5759439468384</v>
       </c>
       <c r="F3" t="n">
-        <v>20.14236111111111</v>
+        <v>20.11458333333333</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>19yr_f_c_kd_080.mp4</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>6.511852223014644</v>
+      </c>
+      <c r="C4" t="n">
+        <v>2.060674157303371</v>
+      </c>
+      <c r="D4" t="n">
+        <v>301.8271484375</v>
+      </c>
+      <c r="E4" t="n">
+        <v>492.5759439468384</v>
+      </c>
+      <c r="F4" t="n">
+        <v>20.74606741573034</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>12yr_m_b_av_006_bq.mp4</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>10.91907606690508</v>
+      </c>
+      <c r="C5" t="n">
+        <v>6.140350877192983</v>
+      </c>
+      <c r="D5" t="n">
+        <v>301.8271484375</v>
+      </c>
+      <c r="E5" t="n">
+        <v>492.5759439468384</v>
+      </c>
+      <c r="F5" t="n">
+        <v>18.1244019138756</v>
       </c>
     </row>
   </sheetData>
@@ -526,12 +570,12 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>10.98565969862315</v>
+        <v>9.682438753222721</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>6.946676587301587</v>
+        <v>5.531283044338374</v>
       </c>
     </row>
     <row r="4">

</xml_diff>